<commit_message>
phương tiện + refactor
</commit_message>
<xml_diff>
--- a/docs/Nhóm 16/01 - Tai lieu du an/1. Ke hoach phat hieu yeu cau BTL (Elicitation)/Raw_Log_BlueMoon.xlsx
+++ b/docs/Nhóm 16/01 - Tai lieu du an/1. Ke hoach phat hieu yeu cau BTL (Elicitation)/Raw_Log_BlueMoon.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\download\Nhóm 16-20260402T212907Z-1-001\Nhóm 16\01 - Tai lieu du an\1. Ke hoach phat hieu yeu cau BTL (Elicitation)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BlueMoon\docs\Nhóm 16\01 - Tai lieu du an\1. Ke hoach phat hieu yeu cau BTL (Elicitation)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5872FC0-AEA0-401E-A81E-677C966D4956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F2682F-A6FC-47AE-A0D2-89D1E8505034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Log" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="157">
   <si>
     <t>RAW LOG — Phần mềm quản lý thu phí chung cư BlueMoon</t>
   </si>
@@ -463,9 +463,6 @@
     <t>Có thể để v2.0 hoặc xem xét lại</t>
   </si>
   <si>
-    <t>Nhóm 6  |  Môn: Nhập môn Công nghệ Phần mềm  |  Trường: SOICT – HUST  |  Phiên bản: v1.0</t>
-  </si>
-  <si>
     <t>RL-025</t>
   </si>
   <si>
@@ -509,6 +506,9 @@
   </si>
   <si>
     <t>Trung bình. Yêu cầu truy vết thông báo. Tính năng v2.0. Phụ thuộc RL-016 (thông báo tự động) chưa làm trong v1.0.</t>
+  </si>
+  <si>
+    <t>Nhóm 16  |  Môn: Nhập môn Công nghệ Phần mềm  |  Trường: SOICT – HUST  |  Phiên bản: v1.0</t>
   </si>
 </sst>
 </file>
@@ -795,14 +795,14 @@
     <xf numFmtId="0" fontId="4" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1119,7 +1119,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="24"/>
@@ -1129,8 +1129,8 @@
       <c r="F1" s="24"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
-        <v>141</v>
+      <c r="A2" s="25" t="s">
+        <v>156</v>
       </c>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
@@ -1495,7 +1495,7 @@
         <v>76</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1532,10 +1532,10 @@
         <v>10</v>
       </c>
       <c r="E22" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>143</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1555,7 +1555,7 @@
         <v>85</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1575,7 +1575,7 @@
         <v>89</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1595,7 +1595,7 @@
         <v>92</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1615,7 +1615,7 @@
         <v>96</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1635,18 +1635,18 @@
         <v>99</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B28" s="17" t="s">
         <v>94</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D28" s="18" t="s">
         <v>88</v>
@@ -1655,7 +1655,7 @@
         <v>105</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1675,7 +1675,7 @@
         <v>102</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1686,16 +1686,16 @@
         <v>94</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D30" s="15" t="s">
         <v>88</v>
       </c>
       <c r="E30" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="F30" s="9" t="s">
         <v>153</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -1739,7 +1739,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="23" t="s">
         <v>110</v>
       </c>
       <c r="B1" s="24"/>

</xml_diff>

<commit_message>
cập nhật tài liệu
</commit_message>
<xml_diff>
--- a/docs/Nhóm 16/01 - Tai lieu du an/1. Ke hoach phat hieu yeu cau BTL (Elicitation)/Raw_Log_BlueMoon.xlsx
+++ b/docs/Nhóm 16/01 - Tai lieu du an/1. Ke hoach phat hieu yeu cau BTL (Elicitation)/Raw_Log_BlueMoon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BlueMoon\docs\Nhóm 16\01 - Tai lieu du an\1. Ke hoach phat hieu yeu cau BTL (Elicitation)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F2682F-A6FC-47AE-A0D2-89D1E8505034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9033744C-0865-42C8-ADAD-BC40482B84B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Log" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="195">
   <si>
     <t>RAW LOG — Phần mềm quản lý thu phí chung cư BlueMoon</t>
   </si>
@@ -81,9 +81,6 @@
     <t>RL-002</t>
   </si>
   <si>
-    <t>Là trưởng ban quản trị, tôi muốn hệ thống phân quyền rõ ràng: kế toán chỉ nhập liệu thu phí, trưởng ban mới được xuất báo cáo và quản lý tài khoản.</t>
-  </si>
-  <si>
     <t>Use Case / User Story (Phân quyền người dùng)</t>
   </si>
   <si>
@@ -291,9 +288,6 @@
     <t>RL-020</t>
   </si>
   <si>
-    <t>Là trưởng ban quản trị, tôi muốn quản lý các khoản thu hộ hàng tháng (điện, nước, internet) theo thông báo từ các công ty cung cấp dịch vụ.</t>
-  </si>
-  <si>
     <t>User Story / Feature (Thu hộ điện – nước – internet) [v2.0]</t>
   </si>
   <si>
@@ -312,9 +306,6 @@
     <t>RL-022</t>
   </si>
   <si>
-    <t>Hệ thống phải hỗ trợ phân quyền ít nhất 2 vai trò: trưởng ban (full access) và kế toán (chỉ nhập liệu, không xuất báo cáo tổng hợp).</t>
-  </si>
-  <si>
     <t>Technical Story / Acceptance Criteria (Phân quyền – Authorization)</t>
   </si>
   <si>
@@ -364,9 +355,6 @@
   </si>
   <si>
     <t>User Story / Feature (Tra cứu phí cá nhân – Cổng cư dân)</t>
-  </si>
-  <si>
-    <t>Thấp. Cải thiện trải nghiệm. Có thể để v2.0.</t>
   </si>
   <si>
     <t>HƯỚNG DẪN SỬ DỤNG RAW LOG</t>
@@ -478,21 +466,6 @@
     <t>Cao. Bảo mật. Bắt buộc có. Liên kết RL-001. Tương đương NFR-001</t>
   </si>
   <si>
-    <t>Cao. Bảo mật. Chi tiết của RL-002.              Tương đương NFR-002</t>
-  </si>
-  <si>
-    <t>Trung bình. Truy vết &amp; bảo mật.                Tương đương NFR-003</t>
-  </si>
-  <si>
-    <t>Trung bình. Hiệu năng.                          Tương đương NFR-004</t>
-  </si>
-  <si>
-    <t>Trung bình. Usability.                             Tương đương NFR-006.</t>
-  </si>
-  <si>
-    <t>Cao. Độ tin cậy.                                          Tương đương NFR-005</t>
-  </si>
-  <si>
     <t>Mã nguồn phải tuân thủ Java Coding Convention và có Javadoc cho các class, method chính.</t>
   </si>
   <si>
@@ -508,14 +481,168 @@
     <t>Trung bình. Yêu cầu truy vết thông báo. Tính năng v2.0. Phụ thuộc RL-016 (thông báo tự động) chưa làm trong v1.0.</t>
   </si>
   <si>
-    <t>Nhóm 16  |  Môn: Nhập môn Công nghệ Phần mềm  |  Trường: SOICT – HUST  |  Phiên bản: v1.0</t>
+    <t>Là trưởng ban quản trị, tôi muốn hệ thống phân quyền rõ ràng: kế toán có toàn quyền nghiệp vụ thu phí, dân cư và xuất báo cáo; trưởng ban có thêm quyền quản lý người dùng, xem nhật ký hệ thống và thùng rác — đây là 3 module duy nhất giới hạn riêng cho trưởng ban.</t>
+  </si>
+  <si>
+    <t>Hệ thống phải hỗ trợ phân quyền ít nhất 2 vai trò: trưởng ban (full access) và kế toán có toàn quyền nghiệp vụ thu phí, dân cư và xuất báo cáo; trưởng ban có thêm quyền quản lý người dùng, xem nhật ký hệ thống và thùng rác — đây là 3 module duy nhất giới hạn riêng cho trưởng ban.</t>
+  </si>
+  <si>
+    <t>Là trưởng ban quản trị, tôi muốn quản lý các khoản thu hộ hàng tháng (điện, nước, internet, gas) dùng dữ liệu hóa đơn mô phỏng (SimulationDataService) do dự án không có quyền truy cập API thật từ nhà cung cấp (EVN, Hawaco, nhà mạng...), quản lý qua entity riêng HoaDonThuHo tại /thu-ho, tách biệt hoàn toàn khỏi module khoản thu chính.</t>
+  </si>
+  <si>
+    <t>Từ chối / Out of Scope. Hệ thống là cổng nội bộ khép kín (Internal Portal), cư dân không có tài khoản đăng nhập theo quyết định tại Project Charter mục 4.5. Không triển khai ở cả v1.0 và v2.0.</t>
+  </si>
+  <si>
+    <t>RL-029</t>
+  </si>
+  <si>
+    <t>Là kế toán, tôi muốn quản lý phương tiện (xe máy/ô tô) của từng hộ gia đình, kiểm tra trùng biển số.</t>
+  </si>
+  <si>
+    <t>User Story / Feature (Quản lý phương tiện)</t>
+  </si>
+  <si>
+    <t>Cao. Tương đương RL-025 trong Kế hoạch Scrum.</t>
+  </si>
+  <si>
+    <t>RL-030</t>
+  </si>
+  <si>
+    <t>User Story / Feature (Mẫu khoản thu định kỳ)</t>
+  </si>
+  <si>
+    <t>Cao. Tương đương RL-026 trong Kế hoạch Scrum.</t>
+  </si>
+  <si>
+    <t>RL-031</t>
+  </si>
+  <si>
+    <t>Hệ thống phải lưu lịch sử mọi lần gửi email thông báo.</t>
+  </si>
+  <si>
+    <t>Technical Story (Lịch sử email)</t>
+  </si>
+  <si>
+    <t>RL-032</t>
+  </si>
+  <si>
+    <t>User Story / Feature (Quản lý người dùng)</t>
+  </si>
+  <si>
+    <t>Cao. Tương đương RL-028 trong Kế hoạch Scrum.</t>
+  </si>
+  <si>
+    <t>RL-033</t>
+  </si>
+  <si>
+    <t>Là kế toán, tôi muốn quản lý danh mục loại khoản thu để phân loại các khoản phí.</t>
+  </si>
+  <si>
+    <t>User Story / Feature (Loại khoản thu)</t>
+  </si>
+  <si>
+    <t>RL-034</t>
+  </si>
+  <si>
+    <t>Technical Story (Auto-apply khoản thu)</t>
+  </si>
+  <si>
+    <t>Cao. Tương đương RL-030 trong Kế hoạch Scrum.</t>
+  </si>
+  <si>
+    <t>RL-035</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn xem tổng hợp trạng thái thu phí của tất cả hộ trên 1 màn hình.</t>
+  </si>
+  <si>
+    <t>User Story / Feature (Theo dõi tổng hợp)</t>
+  </si>
+  <si>
+    <t>RL-036</t>
+  </si>
+  <si>
+    <t>Hệ thống phải hỗ trợ migration cơ sở dữ liệu, gộp vào 1 file schema duy nhất.</t>
+  </si>
+  <si>
+    <t>Technical Story (DB Migration)</t>
+  </si>
+  <si>
+    <t>RL-037</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn khôi phục hoặc xóa vĩnh viễn dữ liệu hộ gia đình/khoản thu đã xóa mềm.</t>
+  </si>
+  <si>
+    <t>User Story / Feature (Thùng rác)</t>
+  </si>
+  <si>
+    <t>Ô xám nhạt – Từ chối / Out of Scope</t>
+  </si>
+  <si>
+    <t>Yêu cầu bị từ chối, không triển khai ở cả v1.0 và v2.0</t>
+  </si>
+  <si>
+    <t>Cao. Bảo mật. Chi tiết của RL-002.              
+Tương đương NFR-002</t>
+  </si>
+  <si>
+    <t>Trung bình. Truy vết &amp; bảo mật.                
+Tương đương NFR-003</t>
+  </si>
+  <si>
+    <t>Trung bình. Hiệu năng.                          
+Tương đương NFR-004</t>
+  </si>
+  <si>
+    <t>Trung bình. Usability.                             
+Tương đương NFR-006.</t>
+  </si>
+  <si>
+    <t>Cao. Độ tin cậy.                                          
+Tương đương NFR-005</t>
+  </si>
+  <si>
+    <t>Trung bình. Tương đương RL-027 trong Kế hoạch 
+Scrum, nội dung liên quan tới RL-017.</t>
+  </si>
+  <si>
+    <t>Trung bình. Tương đương RL-029 trong Kế hoạch 
+Scrum.</t>
+  </si>
+  <si>
+    <t>Hệ thống phải tự động tạo bản ghi thanh toán CON_NO cho mọi hộ khi tạo một khoản 
+thu bắt buộc mới.</t>
+  </si>
+  <si>
+    <t>Hệ thống phải tự động sinh khoản thu định kỳ mỗi tháng theo mẫu đã thiết lập (ngày 
+28 hàng tháng).</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn quản lý tài khoản người dùng hệ thống (thêm/sửa/khóa/phân 
+quyền).</t>
+  </si>
+  <si>
+    <t>Trung bình. Chi tiết của RL-009. Tương đương 
+RL-031 trong Kế hoạch Scrum.</t>
+  </si>
+  <si>
+    <t>Trung bình. Tương đương RL-032 trong Kế hoạch 
+Scrum.</t>
+  </si>
+  <si>
+    <t>Trung bình. Tương đương RL-033 trong Kế hoạch 
+Scrum.</t>
+  </si>
+  <si>
+    <t>Nhóm 16  |  Môn: Nhập môn Công nghệ Phần mềm  |  Trường: SOICT – HUST  |  Phiên bản: v1.0 + v2.0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -600,8 +727,52 @@
       <family val="2"/>
       <charset val="163"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1A5276"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1A5276"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF7D6608"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -660,17 +831,54 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCCCC"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF4FB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6E4F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF8E1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3CD"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -723,11 +931,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA0A0A0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFA0A0A0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFA0A0A0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA0A0A0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFA0A0A0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFA0A0A0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA0A0A0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFA0A0A0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -783,27 +1028,139 @@
     <xf numFmtId="0" fontId="8" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1105,9 +1462,31 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{D5EDF202-C03D-4661-98BB-B9DFB482CC65}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;6742418f-f29f-4761-a222-c1e0b165da3a&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1115,28 +1494,28 @@
     <col min="3" max="3" width="68" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="6" max="6" width="36" customWidth="1"/>
+    <col min="6" max="6" width="40.296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
-        <v>156</v>
-      </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
+      <c r="A2" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
     </row>
     <row r="3" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1186,536 +1565,716 @@
         <v>8</v>
       </c>
       <c r="C5" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="7" t="s">
+      <c r="F5" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="9" t="s">
         <v>19</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="7" t="s">
+      <c r="F7" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="7" t="s">
+      <c r="D11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" s="7" t="s">
+      <c r="F11" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>8</v>
       </c>
       <c r="C13" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" s="7" t="s">
+      <c r="F13" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="5" t="s">
         <v>52</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="7" t="s">
+      <c r="F15" s="5" t="s">
         <v>56</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>8</v>
       </c>
       <c r="C17" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D17" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" s="7" t="s">
+      <c r="F17" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C18" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>68</v>
-      </c>
       <c r="F18" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>8</v>
       </c>
       <c r="C19" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E19" s="7" t="s">
+      <c r="F19" s="9" t="s">
         <v>71</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C20" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="D20" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="E20" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="E20" s="11" t="s">
-        <v>76</v>
-      </c>
       <c r="F20" s="9" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B21" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="7" t="s">
+      <c r="D21" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="D21" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E21" s="7" t="s">
+      <c r="F21" s="5" t="s">
         <v>79</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>8</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>84</v>
+        <v>149</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B24" s="14" t="s">
         <v>8</v>
       </c>
       <c r="C24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="E24" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="D24" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="E24" s="14" t="s">
-        <v>89</v>
-      </c>
       <c r="F24" s="5" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B25" s="17" t="s">
         <v>8</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>91</v>
+        <v>148</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>146</v>
+        <v>181</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="E26" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="B26" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="D26" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="E26" s="14" t="s">
-        <v>96</v>
-      </c>
       <c r="F26" s="9" t="s">
-        <v>147</v>
+        <v>182</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E27" s="17" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>148</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>149</v>
+        <v>184</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B29" s="17" t="s">
         <v>8</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>150</v>
+        <v>185</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="B30" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="91.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="B30" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C30" s="14" t="s">
+      <c r="B31" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="C31" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="D31" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="F31" s="30" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="31" t="s">
         <v>151</v>
       </c>
-      <c r="D30" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="E30" s="14" t="s">
+      <c r="B32" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="F30" s="9" t="s">
+      <c r="D32" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" s="33" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="F31" s="19" t="s">
-        <v>109</v>
+      <c r="F32" s="29" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" s="51" customFormat="1" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="48" t="s">
+        <v>155</v>
+      </c>
+      <c r="B33" s="49" t="s">
+        <v>91</v>
+      </c>
+      <c r="C33" s="63" t="s">
+        <v>189</v>
+      </c>
+      <c r="D33" s="52" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="F33" s="50" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="59.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="37" t="s">
+        <v>158</v>
+      </c>
+      <c r="B34" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="C34" s="57" t="s">
+        <v>159</v>
+      </c>
+      <c r="D34" s="53" t="s">
+        <v>86</v>
+      </c>
+      <c r="E34" s="57" t="s">
+        <v>160</v>
+      </c>
+      <c r="F34" s="61" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="47.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="B35" s="39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35" s="62" t="s">
+        <v>190</v>
+      </c>
+      <c r="D35" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" s="58" t="s">
+        <v>162</v>
+      </c>
+      <c r="F35" s="50" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="55.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="35" t="s">
+        <v>164</v>
+      </c>
+      <c r="B36" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="C36" s="49" t="s">
+        <v>165</v>
+      </c>
+      <c r="D36" s="52" t="s">
+        <v>10</v>
+      </c>
+      <c r="E36" s="49" t="s">
+        <v>166</v>
+      </c>
+      <c r="F36" s="61" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="52.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="41" t="s">
+        <v>167</v>
+      </c>
+      <c r="B37" s="39" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" s="62" t="s">
+        <v>188</v>
+      </c>
+      <c r="D37" s="54" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" s="58" t="s">
+        <v>168</v>
+      </c>
+      <c r="F37" s="50" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="58.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="35" t="s">
+        <v>170</v>
+      </c>
+      <c r="B38" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" s="49" t="s">
+        <v>171</v>
+      </c>
+      <c r="D38" s="52" t="s">
+        <v>10</v>
+      </c>
+      <c r="E38" s="49" t="s">
+        <v>172</v>
+      </c>
+      <c r="F38" s="61" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="43" t="s">
+        <v>173</v>
+      </c>
+      <c r="B39" s="42" t="s">
+        <v>91</v>
+      </c>
+      <c r="C39" s="59" t="s">
+        <v>174</v>
+      </c>
+      <c r="D39" s="55" t="s">
+        <v>86</v>
+      </c>
+      <c r="E39" s="59" t="s">
+        <v>175</v>
+      </c>
+      <c r="F39" s="61" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="64.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="B40" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="C40" s="60" t="s">
+        <v>177</v>
+      </c>
+      <c r="D40" s="56" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" s="60" t="s">
+        <v>178</v>
+      </c>
+      <c r="F40" s="64" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -1730,7 +2289,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1739,156 +2298,165 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="C3" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="B2" s="20" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C4" s="20" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="21" t="s">
+    <row r="5" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C5" s="20" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="21" t="s">
+    <row r="6" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C6" s="20" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="21" t="s">
+    <row r="7" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="B7" s="20" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="21" t="s">
+      <c r="C7" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="C6" s="21" t="s">
+    </row>
+    <row r="8" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="20" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
+      <c r="C8" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="B7" s="21" t="s">
+    </row>
+    <row r="9" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+    </row>
+    <row r="10" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="B10" s="21" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="21" t="s">
+      <c r="C10" s="21"/>
+    </row>
+    <row r="11" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="B11" s="20" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="21"/>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-    </row>
-    <row r="10" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="22" t="s">
+      <c r="C11" s="20"/>
+    </row>
+    <row r="12" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B12" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="C10" s="22"/>
-    </row>
-    <row r="11" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="21" t="s">
+      <c r="C12" s="20"/>
+    </row>
+    <row r="13" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B13" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="C11" s="21"/>
-    </row>
-    <row r="12" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
+      <c r="C13" s="20"/>
+    </row>
+    <row r="14" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B14" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="C12" s="21"/>
-    </row>
-    <row r="13" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
+      <c r="C14" s="20"/>
+    </row>
+    <row r="15" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B15" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="C13" s="21"/>
-    </row>
-    <row r="14" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="21" t="s">
+      <c r="C15" s="20"/>
+    </row>
+    <row r="16" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="44" t="s">
         <v>135</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B16" s="44" t="s">
         <v>136</v>
       </c>
-      <c r="C14" s="21"/>
-    </row>
-    <row r="15" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="C15" s="21"/>
-    </row>
-    <row r="16" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="B16" s="21" t="s">
-        <v>140</v>
-      </c>
-      <c r="C16" s="21"/>
+      <c r="C16" s="44"/>
+    </row>
+    <row r="17" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A17" s="45" t="s">
+        <v>179</v>
+      </c>
+      <c r="B17" s="46" t="s">
+        <v>180</v>
+      </c>
+      <c r="C17" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>